<commit_message>
Hindalco: update PDFs & Excel (2026-02-16 03:25:47 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F250"/>
+  <dimension ref="A1:F251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -481,23 +481,23 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2431,23 +2431,23 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2461,23 +2461,23 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2761,23 +2761,23 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2851,23 +2851,23 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2881,23 +2881,23 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3061,23 +3061,23 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3571,23 +3571,23 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3691,23 +3691,23 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3721,23 +3721,23 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3811,23 +3811,23 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5671,23 +5671,23 @@
         </is>
       </c>
       <c r="D175" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E175" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F175" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5701,23 +5701,23 @@
         </is>
       </c>
       <c r="D176" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E176" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F176" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5791,23 +5791,23 @@
         </is>
       </c>
       <c r="D179" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E179" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5881,23 +5881,23 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E182" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5911,23 +5911,23 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E183" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6841,23 +6841,23 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F214" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6901,23 +6901,23 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F216" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7081,23 +7081,23 @@
         </is>
       </c>
       <c r="D222" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E222" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F222" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7261,23 +7261,23 @@
         </is>
       </c>
       <c r="D228" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E228" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F228" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7351,23 +7351,23 @@
         </is>
       </c>
       <c r="D231" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E231" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F231" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7471,23 +7471,23 @@
         </is>
       </c>
       <c r="D235" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E235" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F235" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7531,23 +7531,23 @@
         </is>
       </c>
       <c r="D237" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E237" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F237" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7561,23 +7561,23 @@
         </is>
       </c>
       <c r="D238" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E238" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F238" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7591,23 +7591,23 @@
         </is>
       </c>
       <c r="D239" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E239" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F239" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7741,23 +7741,23 @@
         </is>
       </c>
       <c r="D244" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E244" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F244" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7771,23 +7771,23 @@
         </is>
       </c>
       <c r="D245" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E245" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F245" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7929,6 +7929,36 @@
         </is>
       </c>
       <c r="F250" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B251" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C251" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E251" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F251" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8185,6 +8215,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F248" r:id="rId247"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F249" r:id="rId248"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId250"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-17 03:20:15 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F251"/>
+  <dimension ref="A1:F252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2341,23 +2341,23 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2461,23 +2461,23 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2491,23 +2491,23 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2671,23 +2671,23 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2791,23 +2791,23 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2881,23 +2881,23 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3091,23 +3091,23 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3631,23 +3631,23 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3721,23 +3721,23 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3781,23 +3781,23 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5521,23 +5521,23 @@
         </is>
       </c>
       <c r="D170" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5701,23 +5701,23 @@
         </is>
       </c>
       <c r="D176" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E176" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F176" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5731,23 +5731,23 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E177" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F177" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5821,23 +5821,23 @@
         </is>
       </c>
       <c r="D180" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E180" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5911,23 +5911,23 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E183" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5941,23 +5941,23 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E184" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6781,23 +6781,23 @@
         </is>
       </c>
       <c r="D212" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F212" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6871,23 +6871,23 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6931,23 +6931,23 @@
         </is>
       </c>
       <c r="D217" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E217" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F217" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7111,23 +7111,23 @@
         </is>
       </c>
       <c r="D223" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E223" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F223" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7291,23 +7291,23 @@
         </is>
       </c>
       <c r="D229" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E229" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F229" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7381,23 +7381,23 @@
         </is>
       </c>
       <c r="D232" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E232" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F232" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7501,23 +7501,23 @@
         </is>
       </c>
       <c r="D236" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E236" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F236" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7561,23 +7561,23 @@
         </is>
       </c>
       <c r="D238" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E238" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F238" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7591,23 +7591,23 @@
         </is>
       </c>
       <c r="D239" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E239" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F239" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7621,23 +7621,23 @@
         </is>
       </c>
       <c r="D240" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E240" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F240" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7771,23 +7771,23 @@
         </is>
       </c>
       <c r="D245" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E245" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F245" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7801,23 +7801,23 @@
         </is>
       </c>
       <c r="D246" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E246" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F246" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7959,6 +7959,36 @@
         </is>
       </c>
       <c r="F251" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B252" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C252" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E252" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F252" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8216,6 +8246,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F249" r:id="rId248"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId249"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId251"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-17 07:31:11 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-18 03:23:45 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F252"/>
+  <dimension ref="A1:F253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2371,23 +2371,23 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2491,23 +2491,23 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2701,23 +2701,23 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2821,23 +2821,23 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3031,23 +3031,23 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3631,23 +3631,23 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3661,23 +3661,23 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3781,23 +3781,23 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3811,23 +3811,23 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4261,23 +4261,23 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4711,23 +4711,23 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5551,23 +5551,23 @@
         </is>
       </c>
       <c r="D171" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E171" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F171" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5731,23 +5731,23 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E177" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F177" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5761,23 +5761,23 @@
         </is>
       </c>
       <c r="D178" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E178" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F178" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5851,23 +5851,23 @@
         </is>
       </c>
       <c r="D181" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E181" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5941,23 +5941,23 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E184" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5971,23 +5971,23 @@
         </is>
       </c>
       <c r="D185" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E185" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6811,23 +6811,23 @@
         </is>
       </c>
       <c r="D213" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F213" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6901,23 +6901,23 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F216" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6961,23 +6961,23 @@
         </is>
       </c>
       <c r="D218" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E218" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F218" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7141,23 +7141,23 @@
         </is>
       </c>
       <c r="D224" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E224" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F224" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7321,23 +7321,23 @@
         </is>
       </c>
       <c r="D230" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E230" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F230" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7411,23 +7411,23 @@
         </is>
       </c>
       <c r="D233" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E233" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F233" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7531,23 +7531,23 @@
         </is>
       </c>
       <c r="D237" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E237" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F237" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7591,23 +7591,23 @@
         </is>
       </c>
       <c r="D239" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E239" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F239" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7621,23 +7621,23 @@
         </is>
       </c>
       <c r="D240" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E240" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F240" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7651,23 +7651,23 @@
         </is>
       </c>
       <c r="D241" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E241" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F241" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7801,23 +7801,23 @@
         </is>
       </c>
       <c r="D246" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E246" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F246" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7831,23 +7831,23 @@
         </is>
       </c>
       <c r="D247" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E247" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F247" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7989,6 +7989,36 @@
         </is>
       </c>
       <c r="F252" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B253" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C253" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E253" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F253" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8247,6 +8277,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId249"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId250"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId252"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-18 07:32:00 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-19 03:22:24 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F253"/>
+  <dimension ref="A1:F254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2401,23 +2401,23 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2731,23 +2731,23 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2851,23 +2851,23 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3031,23 +3031,23 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3061,23 +3061,23 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3481,23 +3481,23 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3661,23 +3661,23 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3691,23 +3691,23 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3781,23 +3781,23 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3811,23 +3811,23 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3901,23 +3901,23 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4291,23 +4291,23 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4621,23 +4621,23 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5581,23 +5581,23 @@
         </is>
       </c>
       <c r="D172" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E172" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F172" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5761,23 +5761,23 @@
         </is>
       </c>
       <c r="D178" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E178" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F178" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5791,23 +5791,23 @@
         </is>
       </c>
       <c r="D179" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E179" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5881,23 +5881,23 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E182" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5971,23 +5971,23 @@
         </is>
       </c>
       <c r="D185" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E185" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6001,23 +6001,23 @@
         </is>
       </c>
       <c r="D186" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E186" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6841,23 +6841,23 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F214" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6931,23 +6931,23 @@
         </is>
       </c>
       <c r="D217" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E217" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F217" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -6991,23 +6991,23 @@
         </is>
       </c>
       <c r="D219" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E219" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F219" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7171,23 +7171,23 @@
         </is>
       </c>
       <c r="D225" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E225" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F225" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7351,23 +7351,23 @@
         </is>
       </c>
       <c r="D231" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E231" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F231" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7441,23 +7441,23 @@
         </is>
       </c>
       <c r="D234" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E234" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F234" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7561,23 +7561,23 @@
         </is>
       </c>
       <c r="D238" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E238" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F238" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7621,23 +7621,23 @@
         </is>
       </c>
       <c r="D240" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E240" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F240" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7651,23 +7651,23 @@
         </is>
       </c>
       <c r="D241" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E241" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F241" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7681,23 +7681,23 @@
         </is>
       </c>
       <c r="D242" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E242" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F242" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7831,23 +7831,23 @@
         </is>
       </c>
       <c r="D247" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E247" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F247" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7861,23 +7861,23 @@
         </is>
       </c>
       <c r="D248" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E248" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F248" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8019,6 +8019,36 @@
         </is>
       </c>
       <c r="F253" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B254" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C254" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E254" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F254" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8278,6 +8308,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId250"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId251"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId253"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-19 07:31:17 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-20 03:17:25 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F254"/>
+  <dimension ref="A1:F255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2341,23 +2341,23 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2431,23 +2431,23 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2671,23 +2671,23 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2761,23 +2761,23 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2881,23 +2881,23 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3031,23 +3031,23 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3061,23 +3061,23 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3091,23 +3091,23 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3481,23 +3481,23 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3511,23 +3511,23 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3691,23 +3691,23 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3721,23 +3721,23 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3811,23 +3811,23 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4321,23 +4321,23 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5611,23 +5611,23 @@
         </is>
       </c>
       <c r="D173" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E173" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5791,23 +5791,23 @@
         </is>
       </c>
       <c r="D179" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E179" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5821,23 +5821,23 @@
         </is>
       </c>
       <c r="D180" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E180" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5911,23 +5911,23 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E183" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6001,23 +6001,23 @@
         </is>
       </c>
       <c r="D186" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E186" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6031,23 +6031,23 @@
         </is>
       </c>
       <c r="D187" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E187" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6871,23 +6871,23 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6961,23 +6961,23 @@
         </is>
       </c>
       <c r="D218" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E218" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F218" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7021,23 +7021,23 @@
         </is>
       </c>
       <c r="D220" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E220" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F220" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7201,23 +7201,23 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E226" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F226" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7381,23 +7381,23 @@
         </is>
       </c>
       <c r="D232" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E232" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F232" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7471,23 +7471,23 @@
         </is>
       </c>
       <c r="D235" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E235" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F235" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7591,23 +7591,23 @@
         </is>
       </c>
       <c r="D239" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E239" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F239" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7651,23 +7651,23 @@
         </is>
       </c>
       <c r="D241" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E241" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F241" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7681,23 +7681,23 @@
         </is>
       </c>
       <c r="D242" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E242" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F242" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7711,23 +7711,23 @@
         </is>
       </c>
       <c r="D243" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E243" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F243" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7861,23 +7861,23 @@
         </is>
       </c>
       <c r="D248" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E248" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F248" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7891,23 +7891,23 @@
         </is>
       </c>
       <c r="D249" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E249" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F249" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8049,6 +8049,36 @@
         </is>
       </c>
       <c r="F254" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B255" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C255" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E255" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F255" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8309,6 +8339,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId251"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId252"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId254"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-21 03:08:34 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F255"/>
+  <dimension ref="A1:F256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2371,23 +2371,23 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2461,23 +2461,23 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2671,23 +2671,23 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2701,23 +2701,23 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2791,23 +2791,23 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3031,23 +3031,23 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3061,23 +3061,23 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3091,23 +3091,23 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3511,23 +3511,23 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3541,23 +3541,23 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3721,23 +3721,23 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3901,23 +3901,23 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4261,23 +4261,23 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5641,23 +5641,23 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E174" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5821,23 +5821,23 @@
         </is>
       </c>
       <c r="D180" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E180" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5851,23 +5851,23 @@
         </is>
       </c>
       <c r="D181" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E181" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5941,23 +5941,23 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E184" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6031,23 +6031,23 @@
         </is>
       </c>
       <c r="D187" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E187" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6781,23 +6781,23 @@
         </is>
       </c>
       <c r="D212" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F212" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6901,23 +6901,23 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F216" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -6991,23 +6991,23 @@
         </is>
       </c>
       <c r="D219" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E219" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F219" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7051,23 +7051,23 @@
         </is>
       </c>
       <c r="D221" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E221" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F221" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7231,23 +7231,23 @@
         </is>
       </c>
       <c r="D227" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E227" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F227" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7411,23 +7411,23 @@
         </is>
       </c>
       <c r="D233" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E233" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F233" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7501,23 +7501,23 @@
         </is>
       </c>
       <c r="D236" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E236" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F236" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7621,23 +7621,23 @@
         </is>
       </c>
       <c r="D240" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E240" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F240" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7681,23 +7681,23 @@
         </is>
       </c>
       <c r="D242" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E242" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F242" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7711,23 +7711,23 @@
         </is>
       </c>
       <c r="D243" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E243" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F243" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7741,23 +7741,23 @@
         </is>
       </c>
       <c r="D244" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E244" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F244" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7891,23 +7891,23 @@
         </is>
       </c>
       <c r="D249" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E249" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F249" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7921,23 +7921,23 @@
         </is>
       </c>
       <c r="D250" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E250" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F250" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8079,6 +8079,36 @@
         </is>
       </c>
       <c r="F255" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B256" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C256" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E256" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F256" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8340,6 +8370,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId252"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId253"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId255"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-21 07:05:17 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-22 03:21:53 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F256"/>
+  <dimension ref="A1:F257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2401,23 +2401,23 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2491,23 +2491,23 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2701,23 +2701,23 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2731,23 +2731,23 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2821,23 +2821,23 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3031,23 +3031,23 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3061,23 +3061,23 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3091,23 +3091,23 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3481,23 +3481,23 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3541,23 +3541,23 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3571,23 +3571,23 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3781,23 +3781,23 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3901,23 +3901,23 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4291,23 +4291,23 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4711,23 +4711,23 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5671,23 +5671,23 @@
         </is>
       </c>
       <c r="D175" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E175" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F175" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5851,23 +5851,23 @@
         </is>
       </c>
       <c r="D181" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E181" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5881,23 +5881,23 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E182" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5971,23 +5971,23 @@
         </is>
       </c>
       <c r="D185" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E185" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6811,23 +6811,23 @@
         </is>
       </c>
       <c r="D213" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F213" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6931,23 +6931,23 @@
         </is>
       </c>
       <c r="D217" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E217" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F217" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7021,23 +7021,23 @@
         </is>
       </c>
       <c r="D220" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E220" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F220" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7081,23 +7081,23 @@
         </is>
       </c>
       <c r="D222" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E222" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F222" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7261,23 +7261,23 @@
         </is>
       </c>
       <c r="D228" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E228" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F228" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7441,23 +7441,23 @@
         </is>
       </c>
       <c r="D234" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E234" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F234" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7531,23 +7531,23 @@
         </is>
       </c>
       <c r="D237" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E237" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F237" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7651,23 +7651,23 @@
         </is>
       </c>
       <c r="D241" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E241" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F241" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7711,23 +7711,23 @@
         </is>
       </c>
       <c r="D243" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E243" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F243" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7741,23 +7741,23 @@
         </is>
       </c>
       <c r="D244" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E244" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F244" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7771,23 +7771,23 @@
         </is>
       </c>
       <c r="D245" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E245" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F245" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7921,23 +7921,23 @@
         </is>
       </c>
       <c r="D250" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E250" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F250" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7951,23 +7951,23 @@
         </is>
       </c>
       <c r="D251" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E251" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F251" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8109,6 +8109,36 @@
         </is>
       </c>
       <c r="F256" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B257" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C257" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E257" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F257" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8371,6 +8401,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId253"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId254"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId256"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-23 03:25:36 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F257"/>
+  <dimension ref="A1:F258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2341,23 +2341,23 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2431,23 +2431,23 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2671,23 +2671,23 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2731,23 +2731,23 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2761,23 +2761,23 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2851,23 +2851,23 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3061,23 +3061,23 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3091,23 +3091,23 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3481,23 +3481,23 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3511,23 +3511,23 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3571,23 +3571,23 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3781,23 +3781,23 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3811,23 +3811,23 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3901,23 +3901,23 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4321,23 +4321,23 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5701,23 +5701,23 @@
         </is>
       </c>
       <c r="D176" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E176" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F176" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5881,23 +5881,23 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E182" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5911,23 +5911,23 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E183" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6001,23 +6001,23 @@
         </is>
       </c>
       <c r="D186" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E186" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6841,23 +6841,23 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F214" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6961,23 +6961,23 @@
         </is>
       </c>
       <c r="D218" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E218" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F218" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7051,23 +7051,23 @@
         </is>
       </c>
       <c r="D221" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E221" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F221" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7111,23 +7111,23 @@
         </is>
       </c>
       <c r="D223" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E223" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F223" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7291,23 +7291,23 @@
         </is>
       </c>
       <c r="D229" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E229" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F229" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7471,23 +7471,23 @@
         </is>
       </c>
       <c r="D235" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E235" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F235" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7561,23 +7561,23 @@
         </is>
       </c>
       <c r="D238" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E238" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F238" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7681,23 +7681,23 @@
         </is>
       </c>
       <c r="D242" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E242" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F242" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7741,23 +7741,23 @@
         </is>
       </c>
       <c r="D244" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E244" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F244" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7771,23 +7771,23 @@
         </is>
       </c>
       <c r="D245" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E245" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F245" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7801,23 +7801,23 @@
         </is>
       </c>
       <c r="D246" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E246" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F246" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7951,23 +7951,23 @@
         </is>
       </c>
       <c r="D251" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E251" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F251" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7981,23 +7981,23 @@
         </is>
       </c>
       <c r="D252" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E252" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F252" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8139,6 +8139,36 @@
         </is>
       </c>
       <c r="F257" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B258" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C258" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E258" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F258" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8402,6 +8432,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId254"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId255"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F258" r:id="rId257"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-24 03:20:54 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F258"/>
+  <dimension ref="A1:F259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2341,23 +2341,23 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2371,23 +2371,23 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2461,23 +2461,23 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2671,23 +2671,23 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2701,23 +2701,23 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2761,23 +2761,23 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2791,23 +2791,23 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2881,23 +2881,23 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3091,23 +3091,23 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3511,23 +3511,23 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3541,23 +3541,23 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3631,23 +3631,23 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3811,23 +3811,23 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4621,23 +4621,23 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5731,23 +5731,23 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E177" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F177" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5911,23 +5911,23 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E183" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5941,23 +5941,23 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E184" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6031,23 +6031,23 @@
         </is>
       </c>
       <c r="D187" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E187" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6781,23 +6781,23 @@
         </is>
       </c>
       <c r="D212" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F212" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6871,23 +6871,23 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -6991,23 +6991,23 @@
         </is>
       </c>
       <c r="D219" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E219" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F219" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7081,23 +7081,23 @@
         </is>
       </c>
       <c r="D222" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E222" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F222" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7141,23 +7141,23 @@
         </is>
       </c>
       <c r="D224" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E224" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F224" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7321,23 +7321,23 @@
         </is>
       </c>
       <c r="D230" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E230" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F230" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7501,23 +7501,23 @@
         </is>
       </c>
       <c r="D236" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E236" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F236" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7591,23 +7591,23 @@
         </is>
       </c>
       <c r="D239" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E239" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F239" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7711,23 +7711,23 @@
         </is>
       </c>
       <c r="D243" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E243" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F243" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7771,23 +7771,23 @@
         </is>
       </c>
       <c r="D245" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E245" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F245" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7801,23 +7801,23 @@
         </is>
       </c>
       <c r="D246" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E246" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F246" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7831,23 +7831,23 @@
         </is>
       </c>
       <c r="D247" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E247" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F247" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7981,23 +7981,23 @@
         </is>
       </c>
       <c r="D252" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E252" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F252" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8011,23 +8011,23 @@
         </is>
       </c>
       <c r="D253" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E253" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F253" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8169,6 +8169,36 @@
         </is>
       </c>
       <c r="F258" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B259" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C259" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E259" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F259" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8433,6 +8463,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId255"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId256"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F259" r:id="rId258"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-25 03:21:57 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F259"/>
+  <dimension ref="A1:F260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2341,23 +2341,23 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2371,23 +2371,23 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2401,23 +2401,23 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2491,23 +2491,23 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2701,23 +2701,23 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2731,23 +2731,23 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2791,23 +2791,23 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2821,23 +2821,23 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3031,23 +3031,23 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3541,23 +3541,23 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3571,23 +3571,23 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3631,23 +3631,23 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3661,23 +3661,23 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4621,23 +4621,23 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5761,23 +5761,23 @@
         </is>
       </c>
       <c r="D178" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E178" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F178" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5941,23 +5941,23 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E184" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5971,23 +5971,23 @@
         </is>
       </c>
       <c r="D185" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E185" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6811,23 +6811,23 @@
         </is>
       </c>
       <c r="D213" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F213" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6901,23 +6901,23 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F216" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7021,23 +7021,23 @@
         </is>
       </c>
       <c r="D220" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E220" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F220" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7111,23 +7111,23 @@
         </is>
       </c>
       <c r="D223" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E223" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F223" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7171,23 +7171,23 @@
         </is>
       </c>
       <c r="D225" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E225" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F225" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7351,23 +7351,23 @@
         </is>
       </c>
       <c r="D231" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E231" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F231" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7531,23 +7531,23 @@
         </is>
       </c>
       <c r="D237" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E237" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F237" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7621,23 +7621,23 @@
         </is>
       </c>
       <c r="D240" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E240" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F240" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7741,23 +7741,23 @@
         </is>
       </c>
       <c r="D244" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E244" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F244" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7801,23 +7801,23 @@
         </is>
       </c>
       <c r="D246" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E246" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F246" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7831,23 +7831,23 @@
         </is>
       </c>
       <c r="D247" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E247" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F247" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7861,23 +7861,23 @@
         </is>
       </c>
       <c r="D248" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E248" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F248" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8011,23 +8011,23 @@
         </is>
       </c>
       <c r="D253" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E253" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F253" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8041,23 +8041,23 @@
         </is>
       </c>
       <c r="D254" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E254" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F254" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8199,6 +8199,36 @@
         </is>
       </c>
       <c r="F259" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B260" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C260" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E260" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F260" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8464,6 +8494,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId256"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F258" r:id="rId257"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F260" r:id="rId259"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-25 07:32:10 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-26 03:17:46 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F260"/>
+  <dimension ref="A1:F261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2371,23 +2371,23 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2401,23 +2401,23 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2431,23 +2431,23 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2731,23 +2731,23 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2761,23 +2761,23 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2821,23 +2821,23 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2851,23 +2851,23 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3061,23 +3061,23 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3481,23 +3481,23 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3571,23 +3571,23 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3661,23 +3661,23 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3691,23 +3691,23 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3901,23 +3901,23 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5791,23 +5791,23 @@
         </is>
       </c>
       <c r="D179" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E179" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F179" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5971,23 +5971,23 @@
         </is>
       </c>
       <c r="D185" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E185" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6001,23 +6001,23 @@
         </is>
       </c>
       <c r="D186" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E186" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6841,23 +6841,23 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F214" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6931,23 +6931,23 @@
         </is>
       </c>
       <c r="D217" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E217" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F217" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7051,23 +7051,23 @@
         </is>
       </c>
       <c r="D221" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E221" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F221" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7141,23 +7141,23 @@
         </is>
       </c>
       <c r="D224" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E224" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F224" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7201,23 +7201,23 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E226" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F226" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7381,23 +7381,23 @@
         </is>
       </c>
       <c r="D232" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E232" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F232" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7561,23 +7561,23 @@
         </is>
       </c>
       <c r="D238" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E238" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F238" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7651,23 +7651,23 @@
         </is>
       </c>
       <c r="D241" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E241" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F241" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7771,23 +7771,23 @@
         </is>
       </c>
       <c r="D245" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E245" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F245" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7831,23 +7831,23 @@
         </is>
       </c>
       <c r="D247" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E247" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F247" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7861,23 +7861,23 @@
         </is>
       </c>
       <c r="D248" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E248" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F248" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7891,23 +7891,23 @@
         </is>
       </c>
       <c r="D249" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E249" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F249" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8041,23 +8041,23 @@
         </is>
       </c>
       <c r="D254" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E254" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F254" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8071,23 +8071,23 @@
         </is>
       </c>
       <c r="D255" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E255" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F255" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8229,6 +8229,36 @@
         </is>
       </c>
       <c r="F260" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B261" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C261" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E261" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F261" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8495,6 +8525,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F258" r:id="rId257"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F259" r:id="rId258"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId260"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-26 07:31:51 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>330.5</v>
+        <v>333.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>25.02.2026</t>
+          <t>26.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-27 03:14:51 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F261"/>
+  <dimension ref="A1:F262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>330.5</v>
+        <v>333.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>25.02.2026</t>
+          <t>26.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2401,23 +2401,23 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2431,23 +2431,23 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2461,23 +2461,23 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2761,23 +2761,23 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2791,23 +2791,23 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2851,23 +2851,23 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2881,23 +2881,23 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3091,23 +3091,23 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3481,23 +3481,23 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3511,23 +3511,23 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3631,23 +3631,23 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3691,23 +3691,23 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3721,23 +3721,23 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3901,23 +3901,23 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4261,23 +4261,23 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4441,23 +4441,23 @@
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4711,23 +4711,23 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5521,23 +5521,23 @@
         </is>
       </c>
       <c r="D170" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5821,23 +5821,23 @@
         </is>
       </c>
       <c r="D180" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E180" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F180" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6001,23 +6001,23 @@
         </is>
       </c>
       <c r="D186" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E186" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F186" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6031,23 +6031,23 @@
         </is>
       </c>
       <c r="D187" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E187" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6781,23 +6781,23 @@
         </is>
       </c>
       <c r="D212" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F212" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6871,23 +6871,23 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6961,23 +6961,23 @@
         </is>
       </c>
       <c r="D218" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E218" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F218" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7081,23 +7081,23 @@
         </is>
       </c>
       <c r="D222" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E222" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F222" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7171,23 +7171,23 @@
         </is>
       </c>
       <c r="D225" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E225" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F225" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7231,23 +7231,23 @@
         </is>
       </c>
       <c r="D227" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E227" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F227" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7411,23 +7411,23 @@
         </is>
       </c>
       <c r="D233" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E233" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F233" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7591,23 +7591,23 @@
         </is>
       </c>
       <c r="D239" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E239" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F239" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7681,23 +7681,23 @@
         </is>
       </c>
       <c r="D242" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E242" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F242" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7801,23 +7801,23 @@
         </is>
       </c>
       <c r="D246" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E246" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F246" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7861,23 +7861,23 @@
         </is>
       </c>
       <c r="D248" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E248" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F248" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7891,23 +7891,23 @@
         </is>
       </c>
       <c r="D249" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E249" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F249" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7921,23 +7921,23 @@
         </is>
       </c>
       <c r="D250" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E250" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F250" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8071,23 +8071,23 @@
         </is>
       </c>
       <c r="D255" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E255" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F255" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8101,23 +8101,23 @@
         </is>
       </c>
       <c r="D256" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E256" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F256" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8259,6 +8259,36 @@
         </is>
       </c>
       <c r="F261" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B262" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C262" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E262" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F262" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8526,6 +8556,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F259" r:id="rId258"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F260" r:id="rId259"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId261"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-27 07:26:36 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>333.25</v>
+        <v>334.5</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>26.02.2026</t>
+          <t>27.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-02-28 02:58:00 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F262"/>
+  <dimension ref="A1:F263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>333.25</v>
+        <v>334.5</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>26.02.2026</t>
+          <t>27.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>330.5</v>
+        <v>333.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>25.02.2026</t>
+          <t>26.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1277,7 +1277,7 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2431,23 +2431,23 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2461,23 +2461,23 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2491,23 +2491,23 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2671,23 +2671,23 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2791,23 +2791,23 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2821,23 +2821,23 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2881,23 +2881,23 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3481,23 +3481,23 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3511,23 +3511,23 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3541,23 +3541,23 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3631,23 +3631,23 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3661,23 +3661,23 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3721,23 +3721,23 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3931,23 +3931,23 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4291,23 +4291,23 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4471,23 +4471,23 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4711,23 +4711,23 @@
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4891,23 +4891,23 @@
         </is>
       </c>
       <c r="D149" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5521,23 +5521,23 @@
         </is>
       </c>
       <c r="D170" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5551,23 +5551,23 @@
         </is>
       </c>
       <c r="D171" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E171" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F171" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5851,23 +5851,23 @@
         </is>
       </c>
       <c r="D181" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E181" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F181" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6031,23 +6031,23 @@
         </is>
       </c>
       <c r="D187" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E187" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F187" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6421,23 +6421,23 @@
         </is>
       </c>
       <c r="D200" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E200" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F200" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6781,23 +6781,23 @@
         </is>
       </c>
       <c r="D212" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F212" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6811,23 +6811,23 @@
         </is>
       </c>
       <c r="D213" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F213" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6901,23 +6901,23 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F216" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -6991,23 +6991,23 @@
         </is>
       </c>
       <c r="D219" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E219" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F219" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7111,23 +7111,23 @@
         </is>
       </c>
       <c r="D223" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E223" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F223" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7201,23 +7201,23 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E226" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F226" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7261,23 +7261,23 @@
         </is>
       </c>
       <c r="D228" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E228" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F228" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7441,23 +7441,23 @@
         </is>
       </c>
       <c r="D234" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E234" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F234" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7621,23 +7621,23 @@
         </is>
       </c>
       <c r="D240" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E240" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F240" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7711,23 +7711,23 @@
         </is>
       </c>
       <c r="D243" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E243" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F243" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7831,23 +7831,23 @@
         </is>
       </c>
       <c r="D247" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E247" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F247" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7891,23 +7891,23 @@
         </is>
       </c>
       <c r="D249" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E249" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F249" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7921,23 +7921,23 @@
         </is>
       </c>
       <c r="D250" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E250" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F250" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7951,23 +7951,23 @@
         </is>
       </c>
       <c r="D251" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E251" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F251" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8101,23 +8101,23 @@
         </is>
       </c>
       <c r="D256" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E256" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F256" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8131,23 +8131,23 @@
         </is>
       </c>
       <c r="D257" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E257" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F257" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8289,6 +8289,36 @@
         </is>
       </c>
       <c r="F262" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B263" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C263" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E263" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F263" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8557,6 +8587,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F260" r:id="rId259"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId260"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId262"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-03-01 03:27:56 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F263"/>
+  <dimension ref="A1:F264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>333.25</v>
+        <v>334.5</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>26.02.2026</t>
+          <t>27.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>330.5</v>
+        <v>333.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>25.02.2026</t>
+          <t>26.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1561,23 +1561,23 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F38" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2461,23 +2461,23 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2491,23 +2491,23 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2701,23 +2701,23 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2821,23 +2821,23 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2851,23 +2851,23 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3031,23 +3031,23 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3151,23 +3151,23 @@
         </is>
       </c>
       <c r="D91" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3511,23 +3511,23 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3541,23 +3541,23 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3571,23 +3571,23 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3617,7 +3617,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3661,23 +3661,23 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3691,23 +3691,23 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3781,23 +3781,23 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3961,23 +3961,23 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4321,23 +4321,23 @@
         </is>
       </c>
       <c r="D130" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4501,23 +4501,23 @@
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4741,23 +4741,23 @@
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4921,23 +4921,23 @@
         </is>
       </c>
       <c r="D150" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5041,23 +5041,23 @@
         </is>
       </c>
       <c r="D154" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5237,7 +5237,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5551,23 +5551,23 @@
         </is>
       </c>
       <c r="D171" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E171" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F171" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5581,23 +5581,23 @@
         </is>
       </c>
       <c r="D172" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E172" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F172" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5881,23 +5881,23 @@
         </is>
       </c>
       <c r="D182" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E182" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F182" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6061,23 +6061,23 @@
         </is>
       </c>
       <c r="D188" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E188" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F188" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6451,23 +6451,23 @@
         </is>
       </c>
       <c r="D201" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F201" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6557,7 +6557,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6631,23 +6631,23 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E207" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F207" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6811,23 +6811,23 @@
         </is>
       </c>
       <c r="D213" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F213" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6841,23 +6841,23 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F214" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6931,23 +6931,23 @@
         </is>
       </c>
       <c r="D217" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E217" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F217" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7021,23 +7021,23 @@
         </is>
       </c>
       <c r="D220" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E220" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F220" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7141,23 +7141,23 @@
         </is>
       </c>
       <c r="D224" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E224" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F224" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7231,23 +7231,23 @@
         </is>
       </c>
       <c r="D227" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E227" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F227" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7291,23 +7291,23 @@
         </is>
       </c>
       <c r="D229" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E229" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F229" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7471,23 +7471,23 @@
         </is>
       </c>
       <c r="D235" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E235" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F235" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7651,23 +7651,23 @@
         </is>
       </c>
       <c r="D241" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E241" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F241" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7741,23 +7741,23 @@
         </is>
       </c>
       <c r="D244" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E244" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F244" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7861,23 +7861,23 @@
         </is>
       </c>
       <c r="D248" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E248" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F248" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7921,23 +7921,23 @@
         </is>
       </c>
       <c r="D250" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E250" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F250" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7951,23 +7951,23 @@
         </is>
       </c>
       <c r="D251" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E251" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F251" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7981,23 +7981,23 @@
         </is>
       </c>
       <c r="D252" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E252" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F252" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8027,7 +8027,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8131,23 +8131,23 @@
         </is>
       </c>
       <c r="D257" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E257" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F257" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8161,23 +8161,23 @@
         </is>
       </c>
       <c r="D258" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E258" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F258" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8319,6 +8319,36 @@
         </is>
       </c>
       <c r="F263" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B264" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C264" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E264" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F264" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8588,6 +8618,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId260"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId261"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId263"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-03-02 03:16:14 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F264"/>
+  <dimension ref="A1:F265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -481,23 +481,23 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>334.5</v>
+        <v>338.25</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>27.02.2026</t>
+          <t>28.02.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>334.5</v>
+        <v>338.25</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>27.02.2026</t>
+          <t>28.02.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>334.5</v>
+        <v>338.25</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>27.02.2026</t>
+          <t>28.02.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>333.25</v>
+        <v>334.5</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>26.02.2026</t>
+          <t>27.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>330.5</v>
+        <v>333.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>25.02.2026</t>
+          <t>26.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -677,7 +677,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -751,23 +751,23 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -917,7 +917,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1337,7 +1337,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1591,23 +1591,23 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F39" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2011,23 +2011,23 @@
         </is>
       </c>
       <c r="D53" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2491,23 +2491,23 @@
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2597,7 +2597,7 @@
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2731,23 +2731,23 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2851,23 +2851,23 @@
         </is>
       </c>
       <c r="D81" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2881,23 +2881,23 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3017,7 +3017,7 @@
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3061,23 +3061,23 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3181,23 +3181,23 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3271,23 +3271,23 @@
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3437,7 +3437,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3481,23 +3481,23 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3541,23 +3541,23 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3571,23 +3571,23 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3691,23 +3691,23 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3721,23 +3721,23 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3781,23 +3781,23 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3811,23 +3811,23 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3857,7 +3857,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -3991,23 +3991,23 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4111,23 +4111,23 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4217,7 +4217,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4351,23 +4351,23 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4531,23 +4531,23 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4621,23 +4621,23 @@
         </is>
       </c>
       <c r="D140" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4771,23 +4771,23 @@
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4951,23 +4951,23 @@
         </is>
       </c>
       <c r="D151" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5071,23 +5071,23 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5161,23 +5161,23 @@
         </is>
       </c>
       <c r="D158" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5371,23 +5371,23 @@
         </is>
       </c>
       <c r="D165" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5581,23 +5581,23 @@
         </is>
       </c>
       <c r="D172" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E172" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F172" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5611,23 +5611,23 @@
         </is>
       </c>
       <c r="D173" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E173" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5911,23 +5911,23 @@
         </is>
       </c>
       <c r="D183" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E183" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F183" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6091,23 +6091,23 @@
         </is>
       </c>
       <c r="D189" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E189" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F189" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6211,23 +6211,23 @@
         </is>
       </c>
       <c r="D193" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E193" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F193" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6301,23 +6301,23 @@
         </is>
       </c>
       <c r="D196" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E196" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F196" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6377,7 +6377,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6481,23 +6481,23 @@
         </is>
       </c>
       <c r="D202" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F202" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6587,7 +6587,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6661,23 +6661,23 @@
         </is>
       </c>
       <c r="D208" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E208" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F208" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6737,7 +6737,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6841,23 +6841,23 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E214" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F214" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6871,23 +6871,23 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6917,7 +6917,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6961,23 +6961,23 @@
         </is>
       </c>
       <c r="D218" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E218" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F218" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7051,23 +7051,23 @@
         </is>
       </c>
       <c r="D221" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E221" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F221" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7171,23 +7171,23 @@
         </is>
       </c>
       <c r="D225" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E225" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F225" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7261,23 +7261,23 @@
         </is>
       </c>
       <c r="D228" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E228" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F228" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7321,23 +7321,23 @@
         </is>
       </c>
       <c r="D230" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E230" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F230" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7501,23 +7501,23 @@
         </is>
       </c>
       <c r="D236" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E236" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F236" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7681,23 +7681,23 @@
         </is>
       </c>
       <c r="D242" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E242" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F242" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7771,23 +7771,23 @@
         </is>
       </c>
       <c r="D245" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E245" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F245" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7891,23 +7891,23 @@
         </is>
       </c>
       <c r="D249" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E249" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F249" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7951,23 +7951,23 @@
         </is>
       </c>
       <c r="D251" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E251" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F251" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7981,23 +7981,23 @@
         </is>
       </c>
       <c r="D252" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E252" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F252" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8011,23 +8011,23 @@
         </is>
       </c>
       <c r="D253" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E253" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F253" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8057,7 +8057,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8161,23 +8161,23 @@
         </is>
       </c>
       <c r="D258" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E258" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F258" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8191,23 +8191,23 @@
         </is>
       </c>
       <c r="D259" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E259" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F259" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8237,7 +8237,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8349,6 +8349,36 @@
         </is>
       </c>
       <c r="F264" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B265" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C265" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E265" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F265" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8619,6 +8649,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId261"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId262"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId264"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-03-03 03:19:44 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F265"/>
+  <dimension ref="A1:F266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -571,23 +571,23 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>334.5</v>
+        <v>338.25</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>27.02.2026</t>
+          <t>28.02.2026</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>333.25</v>
+        <v>334.5</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>26.02.2026</t>
+          <t>27.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>330.5</v>
+        <v>333.25</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>25.02.2026</t>
+          <t>26.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -781,23 +781,23 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -991,23 +991,23 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1157,7 +1157,7 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1201,23 +1201,23 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1411,23 +1411,23 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1517,7 +1517,7 @@
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1621,23 +1621,23 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F40" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1711,23 +1711,23 @@
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1831,23 +1831,23 @@
         </is>
       </c>
       <c r="D47" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F47" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2041,23 +2041,23 @@
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2117,7 +2117,7 @@
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2251,23 +2251,23 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2341,23 +2341,23 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2521,23 +2521,23 @@
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2671,23 +2671,23 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2761,23 +2761,23 @@
         </is>
       </c>
       <c r="D78" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2881,23 +2881,23 @@
         </is>
       </c>
       <c r="D82" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2957,7 +2957,7 @@
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2971,23 +2971,23 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3091,23 +3091,23 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3137,7 +3137,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3211,23 +3211,23 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3257,7 +3257,7 @@
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3301,23 +3301,23 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3511,23 +3511,23 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3571,23 +3571,23 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3631,23 +3631,23 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3677,7 +3677,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3721,23 +3721,23 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3811,23 +3811,23 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4021,23 +4021,23 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4141,23 +4141,23 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4261,23 +4261,23 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4381,23 +4381,23 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4561,23 +4561,23 @@
         </is>
       </c>
       <c r="D138" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4651,23 +4651,23 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4697,7 +4697,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4801,23 +4801,23 @@
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4877,7 +4877,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4981,23 +4981,23 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5101,23 +5101,23 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5191,23 +5191,23 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5297,7 +5297,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5311,23 +5311,23 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5357,7 +5357,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5401,23 +5401,23 @@
         </is>
       </c>
       <c r="D166" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5461,23 +5461,23 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5537,7 +5537,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5611,23 +5611,23 @@
         </is>
       </c>
       <c r="D173" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E173" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5641,23 +5641,23 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E174" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5941,23 +5941,23 @@
         </is>
       </c>
       <c r="D184" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E184" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F184" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6121,23 +6121,23 @@
         </is>
       </c>
       <c r="D190" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E190" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F190" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6197,7 +6197,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6241,23 +6241,23 @@
         </is>
       </c>
       <c r="D194" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E194" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F194" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6331,23 +6331,23 @@
         </is>
       </c>
       <c r="D197" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E197" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F197" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6511,23 +6511,23 @@
         </is>
       </c>
       <c r="D203" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E203" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F203" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6617,7 +6617,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6691,23 +6691,23 @@
         </is>
       </c>
       <c r="D209" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E209" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F209" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6767,7 +6767,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6781,23 +6781,23 @@
         </is>
       </c>
       <c r="D212" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E212" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F212" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6827,7 +6827,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6871,23 +6871,23 @@
         </is>
       </c>
       <c r="D215" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E215" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F215" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6901,23 +6901,23 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F216" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6947,7 +6947,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -6991,23 +6991,23 @@
         </is>
       </c>
       <c r="D219" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E219" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F219" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7037,7 +7037,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7081,23 +7081,23 @@
         </is>
       </c>
       <c r="D222" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E222" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F222" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7127,7 +7127,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7201,23 +7201,23 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E226" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F226" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7247,7 +7247,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7291,23 +7291,23 @@
         </is>
       </c>
       <c r="D229" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E229" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F229" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7337,7 +7337,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7351,23 +7351,23 @@
         </is>
       </c>
       <c r="D231" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E231" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F231" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7397,7 +7397,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7531,23 +7531,23 @@
         </is>
       </c>
       <c r="D237" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E237" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F237" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7577,7 +7577,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7711,23 +7711,23 @@
         </is>
       </c>
       <c r="D243" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E243" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F243" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7757,7 +7757,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7801,23 +7801,23 @@
         </is>
       </c>
       <c r="D246" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E246" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F246" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7847,7 +7847,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7921,23 +7921,23 @@
         </is>
       </c>
       <c r="D250" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E250" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F250" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7967,7 +7967,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7981,23 +7981,23 @@
         </is>
       </c>
       <c r="D252" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E252" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F252" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8011,23 +8011,23 @@
         </is>
       </c>
       <c r="D253" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E253" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F253" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8041,23 +8041,23 @@
         </is>
       </c>
       <c r="D254" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E254" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F254" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8087,7 +8087,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8191,23 +8191,23 @@
         </is>
       </c>
       <c r="D259" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E259" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F259" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8221,23 +8221,23 @@
         </is>
       </c>
       <c r="D260" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E260" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F260" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8267,7 +8267,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8379,6 +8379,36 @@
         </is>
       </c>
       <c r="F265" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B266" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C266" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E266" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F266" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8650,6 +8680,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId262"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId263"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F266" r:id="rId265"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-03-03 07:13:56 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>338.25</v>
+        <v>346.75</v>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>28.02.2026</t>
+          <t>03.03.2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-march-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-03-04 03:11:05 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F266"/>
+  <dimension ref="A1:F267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -511,23 +511,23 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>338.25</v>
+        <v>346.75</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>28.02.2026</t>
+          <t>03.03.2026</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-march-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -557,7 +557,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -601,23 +601,23 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>334.5</v>
+        <v>338.25</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>27.02.2026</t>
+          <t>28.02.2026</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>333.25</v>
+        <v>334.5</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>26.02.2026</t>
+          <t>27.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>330.5</v>
+        <v>333.25</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>25.02.2026</t>
+          <t>26.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -811,23 +811,23 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -871,23 +871,23 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1231,23 +1231,23 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1397,7 +1397,7 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1441,23 +1441,23 @@
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1651,23 +1651,23 @@
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1741,23 +1741,23 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1861,23 +1861,23 @@
         </is>
       </c>
       <c r="D48" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1921,23 +1921,23 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1997,7 +1997,7 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2071,23 +2071,23 @@
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2161,23 +2161,23 @@
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2237,7 +2237,7 @@
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2281,23 +2281,23 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2341,23 +2341,23 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2371,23 +2371,23 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2417,7 +2417,7 @@
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2551,23 +2551,23 @@
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2657,7 +2657,7 @@
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2701,23 +2701,23 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2791,23 +2791,23 @@
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2837,7 +2837,7 @@
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>13-12-2025</t>
+          <t>14-12-2025</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>12-12-2025</t>
+          <t>13-12-2025</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
@@ -2911,23 +2911,23 @@
         </is>
       </c>
       <c r="D83" s="2" t="n">
-        <v>304.5</v>
+        <v>303</v>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>12.12.2025</t>
+          <t>13.12.2025</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>11-12-2025</t>
+          <t>12-12-2025</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
@@ -2941,23 +2941,23 @@
         </is>
       </c>
       <c r="D84" s="2" t="n">
-        <v>299.5</v>
+        <v>304.5</v>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>10.12.2025</t>
+          <t>12.12.2025</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-december-2025s.pdf</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>10-12-2025</t>
+          <t>11-12-2025</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>09-12-2025</t>
+          <t>10-12-2025</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
@@ -3001,23 +3001,23 @@
         </is>
       </c>
       <c r="D86" s="2" t="n">
-        <v>303</v>
+        <v>299.5</v>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>09.12.2025</t>
+          <t>10.12.2025</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>08-12-2025</t>
+          <t>09-12-2025</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
@@ -3031,23 +3031,23 @@
         </is>
       </c>
       <c r="D87" s="2" t="n">
-        <v>300.5</v>
+        <v>303</v>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>06.12.2025</t>
+          <t>09.12.2025</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>07-12-2025</t>
+          <t>08-12-2025</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
@@ -3077,7 +3077,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>06-12-2025</t>
+          <t>07-12-2025</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>05-12-2025</t>
+          <t>06-12-2025</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
@@ -3121,23 +3121,23 @@
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>298.75</v>
+        <v>300.5</v>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>02.12.2025</t>
+          <t>06.12.2025</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>04-12-2025</t>
+          <t>05-12-2025</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>03-12-2025</t>
+          <t>04-12-2025</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
@@ -3197,7 +3197,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>02-12-2025</t>
+          <t>03-12-2025</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>01-12-2025</t>
+          <t>02-12-2025</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
@@ -3241,23 +3241,23 @@
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>294.5</v>
+        <v>298.75</v>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>29.11.2025</t>
+          <t>02.12.2025</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>30-11-2025</t>
+          <t>01-12-2025</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>29-11-2025</t>
+          <t>30-11-2025</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
@@ -3317,7 +3317,7 @@
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>28-11-2025</t>
+          <t>29-11-2025</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
@@ -3331,23 +3331,23 @@
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>291.75</v>
+        <v>294.5</v>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>28.11.2025</t>
+          <t>29.11.2025</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>27-11-2025</t>
+          <t>28-11-2025</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
@@ -3361,23 +3361,23 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>293.25</v>
+        <v>291.75</v>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>27.11.2025</t>
+          <t>28.11.2025</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>26-11-2025</t>
+          <t>27-11-2025</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
@@ -3391,23 +3391,23 @@
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>288.75</v>
+        <v>293.25</v>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>26.11.2025</t>
+          <t>27.11.2025</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>26-11-2025</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
@@ -3421,23 +3421,23 @@
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>286</v>
+        <v>288.75</v>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>25.11.2025</t>
+          <t>26.11.2025</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
@@ -3451,23 +3451,23 @@
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>22.11.2025</t>
+          <t>25.11.2025</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>23-11-2025</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
@@ -3497,7 +3497,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>22-11-2025</t>
+          <t>23-11-2025</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>21-11-2025</t>
+          <t>22-11-2025</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
@@ -3541,23 +3541,23 @@
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>281.75</v>
+        <v>283</v>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>20.11.2025</t>
+          <t>22.11.2025</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>20-11-2025</t>
+          <t>21-11-2025</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>19-11-2025</t>
+          <t>20-11-2025</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
@@ -3601,23 +3601,23 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>278.25</v>
+        <v>281.75</v>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>19.11.2025</t>
+          <t>20.11.2025</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>18-11-2025</t>
+          <t>19-11-2025</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
@@ -3631,23 +3631,23 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>282.75</v>
+        <v>278.25</v>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>18.11.2025</t>
+          <t>19.11.2025</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>17-11-2025</t>
+          <t>18-11-2025</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
@@ -3661,23 +3661,23 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>286.5</v>
+        <v>282.75</v>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>15.11.2025</t>
+          <t>18.11.2025</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>16-11-2025</t>
+          <t>17-11-2025</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>15-11-2025</t>
+          <t>16-11-2025</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
@@ -3737,7 +3737,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>14-11-2025</t>
+          <t>15-11-2025</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
@@ -3751,23 +3751,23 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>290.5</v>
+        <v>286.5</v>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>14.11.2025</t>
+          <t>15.11.2025</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>13-11-2025</t>
+          <t>14-11-2025</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
@@ -3781,23 +3781,23 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>287.25</v>
+        <v>290.5</v>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>12.11.2025</t>
+          <t>14.11.2025</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>12-11-2025</t>
+          <t>13-11-2025</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>11-11-2025</t>
+          <t>12-11-2025</t>
         </is>
       </c>
       <c r="B114" s="1" t="inlineStr">
@@ -3841,23 +3841,23 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>289.75</v>
+        <v>287.25</v>
       </c>
       <c r="E114" s="1" t="inlineStr">
         <is>
-          <t>11.11.2025</t>
+          <t>12.11.2025</t>
         </is>
       </c>
       <c r="F114" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>10-11-2025</t>
+          <t>11-11-2025</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
@@ -3871,23 +3871,23 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>288.25</v>
+        <v>289.75</v>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>05.11.2025</t>
+          <t>11.11.2025</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>09-11-2025</t>
+          <t>10-11-2025</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
@@ -3917,7 +3917,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>08-11-2025</t>
+          <t>09-11-2025</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>07-11-2025</t>
+          <t>08-11-2025</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
@@ -3977,7 +3977,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>06-11-2025</t>
+          <t>07-11-2025</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>05-11-2025</t>
+          <t>06-11-2025</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
@@ -4037,7 +4037,7 @@
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>04-11-2025</t>
+          <t>05-11-2025</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
@@ -4051,23 +4051,23 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>293.5</v>
+        <v>288.25</v>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>04.11.2025</t>
+          <t>05.11.2025</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>03-11-2025</t>
+          <t>04-11-2025</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
@@ -4081,23 +4081,23 @@
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>291.5</v>
+        <v>293.5</v>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>01.11.2025</t>
+          <t>04.11.2025</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>02-11-2025</t>
+          <t>03-11-2025</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>01-11-2025</t>
+          <t>02-11-2025</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
@@ -4157,7 +4157,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>31-10-2025</t>
+          <t>01-11-2025</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
@@ -4171,23 +4171,23 @@
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>285.5</v>
+        <v>291.5</v>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>31.10.2025</t>
+          <t>01.11.2025</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-november-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>30-10-2025</t>
+          <t>31-10-2025</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
@@ -4201,23 +4201,23 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>290.75</v>
+        <v>285.5</v>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>30.10.2025</t>
+          <t>31.10.2025</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>29-10-2025</t>
+          <t>30-10-2025</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
@@ -4231,23 +4231,23 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>288.75</v>
+        <v>290.75</v>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>28.10.2025</t>
+          <t>30.10.2025</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>28-10-2025</t>
+          <t>29-10-2025</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
@@ -4277,7 +4277,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>27-10-2025</t>
+          <t>28-10-2025</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
@@ -4291,23 +4291,23 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>285.25</v>
+        <v>288.75</v>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>24.10.2025</t>
+          <t>28.10.2025</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>26-10-2025</t>
+          <t>27-10-2025</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
@@ -4337,7 +4337,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>25-10-2025</t>
+          <t>26-10-2025</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>24-10-2025</t>
+          <t>25-10-2025</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>23-10-2025</t>
+          <t>24-10-2025</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
@@ -4411,23 +4411,23 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>279.75</v>
+        <v>285.25</v>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>18.10.2025</t>
+          <t>24.10.2025</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>22-10-2025</t>
+          <t>23-10-2025</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
@@ -4457,7 +4457,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>21-10-2025</t>
+          <t>22-10-2025</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>20-10-2025</t>
+          <t>21-10-2025</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
@@ -4517,7 +4517,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>19-10-2025</t>
+          <t>20-10-2025</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>18-10-2025</t>
+          <t>19-10-2025</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
@@ -4577,7 +4577,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>17-10-2025</t>
+          <t>18-10-2025</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
@@ -4591,23 +4591,23 @@
         </is>
       </c>
       <c r="D139" s="2" t="n">
-        <v>277.25</v>
+        <v>279.75</v>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>15.10.2025</t>
+          <t>18.10.2025</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>16-10-2025</t>
+          <t>17-10-2025</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
@@ -4637,7 +4637,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>15-10-2025</t>
+          <t>16-10-2025</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>15-10-2025</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
@@ -4681,23 +4681,23 @@
         </is>
       </c>
       <c r="D142" s="2" t="n">
-        <v>282.25</v>
+        <v>277.25</v>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>10.10.2025</t>
+          <t>15.10.2025</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>13-10-2025</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>12-10-2025</t>
+          <t>13-10-2025</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
@@ -4757,7 +4757,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>11-10-2025</t>
+          <t>12-10-2025</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>10-10-2025</t>
+          <t>11-10-2025</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>09-10-2025</t>
+          <t>10-10-2025</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
@@ -4831,23 +4831,23 @@
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>278.75</v>
+        <v>282.25</v>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>09.10.2025</t>
+          <t>10.10.2025</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>08-10-2025</t>
+          <t>09-10-2025</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
@@ -4861,23 +4861,23 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>274.25</v>
+        <v>278.75</v>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>04.10.2025</t>
+          <t>09.10.2025</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>07-10-2025</t>
+          <t>08-10-2025</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>06-10-2025</t>
+          <t>07-10-2025</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
@@ -4937,7 +4937,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>05-10-2025</t>
+          <t>06-10-2025</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>04-10-2025</t>
+          <t>05-10-2025</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
@@ -4997,7 +4997,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>03-10-2025</t>
+          <t>04-10-2025</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
@@ -5011,23 +5011,23 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>270.25</v>
+        <v>274.25</v>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>30.09.2025</t>
+          <t>04.10.2025</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-october-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>02-10-2025</t>
+          <t>03-10-2025</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
@@ -5057,7 +5057,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>01-10-2025</t>
+          <t>02-10-2025</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>30-09-2025</t>
+          <t>01-10-2025</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
@@ -5117,7 +5117,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>29-09-2025</t>
+          <t>30-09-2025</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
@@ -5131,23 +5131,23 @@
         </is>
       </c>
       <c r="D157" s="2" t="n">
-        <v>267.25</v>
+        <v>270.25</v>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>27.09.2025</t>
+          <t>30.09.2025</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>28-09-2025</t>
+          <t>29-09-2025</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
@@ -5177,7 +5177,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>27-09-2025</t>
+          <t>28-09-2025</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>26-09-2025</t>
+          <t>27-09-2025</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
@@ -5221,23 +5221,23 @@
         </is>
       </c>
       <c r="D160" s="2" t="n">
-        <v>269</v>
+        <v>267.25</v>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>26.09.2025</t>
+          <t>27.09.2025</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>25-09-2025</t>
+          <t>26-09-2025</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
@@ -5251,23 +5251,23 @@
         </is>
       </c>
       <c r="D161" s="2" t="n">
-        <v>265.5</v>
+        <v>269</v>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>25.09.2025</t>
+          <t>26.09.2025</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>24-09-2025</t>
+          <t>25-09-2025</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
@@ -5281,23 +5281,23 @@
         </is>
       </c>
       <c r="D162" s="2" t="n">
-        <v>267.75</v>
+        <v>265.5</v>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>23.09.2025</t>
+          <t>25.09.2025</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>23-09-2025</t>
+          <t>24-09-2025</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>22-09-2025</t>
+          <t>23-09-2025</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
@@ -5341,23 +5341,23 @@
         </is>
       </c>
       <c r="D164" s="2" t="n">
-        <v>270.5</v>
+        <v>267.75</v>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>20.09.2025</t>
+          <t>23.09.2025</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>21-09-2025</t>
+          <t>22-09-2025</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>20-09-2025</t>
+          <t>21-09-2025</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
@@ -5417,7 +5417,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>19-09-2025</t>
+          <t>20-09-2025</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
@@ -5431,23 +5431,23 @@
         </is>
       </c>
       <c r="D167" s="2" t="n">
-        <v>269</v>
+        <v>270.5</v>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>18.09.2025</t>
+          <t>20.09.2025</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>18-09-2025</t>
+          <t>19-09-2025</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
@@ -5477,7 +5477,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>17-09-2025</t>
+          <t>18-09-2025</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
@@ -5491,23 +5491,23 @@
         </is>
       </c>
       <c r="D169" s="2" t="n">
-        <v>274.25</v>
+        <v>269</v>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>17.09.2025</t>
+          <t>18.09.2025</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>16-09-2025</t>
+          <t>17-09-2025</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
@@ -5521,23 +5521,23 @@
         </is>
       </c>
       <c r="D170" s="2" t="n">
-        <v>272</v>
+        <v>274.25</v>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>13.09.2025</t>
+          <t>17.09.2025</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>15-09-2025</t>
+          <t>16-09-2025</t>
         </is>
       </c>
       <c r="B171" s="1" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>14-09-2025</t>
+          <t>15-09-2025</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
@@ -5597,7 +5597,7 @@
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>13-09-2025</t>
+          <t>14-09-2025</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>12-09-2025</t>
+          <t>13-09-2025</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
@@ -5641,23 +5641,23 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>267.25</v>
+        <v>272</v>
       </c>
       <c r="E174" s="1" t="inlineStr">
         <is>
-          <t>12.09.2025</t>
+          <t>13.09.2025</t>
         </is>
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>12-09-2025</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
@@ -5671,23 +5671,23 @@
         </is>
       </c>
       <c r="D175" s="2" t="n">
-        <v>263</v>
+        <v>267.25</v>
       </c>
       <c r="E175" s="1" t="inlineStr">
         <is>
-          <t>02.09.2025</t>
+          <t>12.09.2025</t>
         </is>
       </c>
       <c r="F175" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
@@ -5717,7 +5717,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>09-09-2025</t>
+          <t>10-09-2025</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>08-09-2025</t>
+          <t>09-09-2025</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
@@ -5777,7 +5777,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>07-09-2025</t>
+          <t>08-09-2025</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>06-09-2025</t>
+          <t>07-09-2025</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
@@ -5837,7 +5837,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>05-09-2025</t>
+          <t>06-09-2025</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>05-09-2025</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
@@ -5897,7 +5897,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>03-09-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>02-09-2025</t>
+          <t>03-09-2025</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
@@ -5957,7 +5957,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>01-09-2025</t>
+          <t>02-09-2025</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
@@ -5971,23 +5971,23 @@
         </is>
       </c>
       <c r="D185" s="2" t="n">
-        <v>261.25</v>
+        <v>263</v>
       </c>
       <c r="E185" s="1" t="inlineStr">
         <is>
-          <t>27.08.2025</t>
+          <t>02.09.2025</t>
         </is>
       </c>
       <c r="F185" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-september-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>31-08-2025</t>
+          <t>01-09-2025</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
@@ -6017,7 +6017,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>30-08-2025</t>
+          <t>31-08-2025</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>29-08-2025</t>
+          <t>30-08-2025</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
@@ -6077,7 +6077,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>28-08-2025</t>
+          <t>29-08-2025</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>27-08-2025</t>
+          <t>28-08-2025</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
@@ -6137,7 +6137,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>26-08-2025</t>
+          <t>27-08-2025</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
@@ -6151,23 +6151,23 @@
         </is>
       </c>
       <c r="D191" s="2" t="n">
-        <v>258.25</v>
+        <v>261.25</v>
       </c>
       <c r="E191" s="1" t="inlineStr">
         <is>
-          <t>26.08.2025</t>
+          <t>27.08.2025</t>
         </is>
       </c>
       <c r="F191" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>25-08-2025</t>
+          <t>26-08-2025</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
@@ -6181,23 +6181,23 @@
         </is>
       </c>
       <c r="D192" s="2" t="n">
-        <v>265</v>
+        <v>258.25</v>
       </c>
       <c r="E192" s="1" t="inlineStr">
         <is>
-          <t>23.08.2025</t>
+          <t>26.08.2025</t>
         </is>
       </c>
       <c r="F192" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>24-08-2025</t>
+          <t>25-08-2025</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>23-08-2025</t>
+          <t>24-08-2025</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
@@ -6257,7 +6257,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>22-08-2025</t>
+          <t>23-08-2025</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
@@ -6271,23 +6271,23 @@
         </is>
       </c>
       <c r="D195" s="2" t="n">
-        <v>262.5</v>
+        <v>265</v>
       </c>
       <c r="E195" s="1" t="inlineStr">
         <is>
-          <t>20.08.2025</t>
+          <t>23.08.2025</t>
         </is>
       </c>
       <c r="F195" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>21-08-2025</t>
+          <t>22-08-2025</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
@@ -6317,7 +6317,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>20-08-2025</t>
+          <t>21-08-2025</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>19-08-2025</t>
+          <t>20-08-2025</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
@@ -6361,23 +6361,23 @@
         </is>
       </c>
       <c r="D198" s="2" t="n">
-        <v>264.75</v>
+        <v>262.5</v>
       </c>
       <c r="E198" s="1" t="inlineStr">
         <is>
-          <t>19.08.2025</t>
+          <t>20.08.2025</t>
         </is>
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>18-08-2025</t>
+          <t>19-08-2025</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
@@ -6391,23 +6391,23 @@
         </is>
       </c>
       <c r="D199" s="2" t="n">
-        <v>269.25</v>
+        <v>264.75</v>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>14.08.2025</t>
+          <t>19.08.2025</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>17-08-2025</t>
+          <t>18-08-2025</t>
         </is>
       </c>
       <c r="B200" s="1" t="inlineStr">
@@ -6437,7 +6437,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>16-08-2025</t>
+          <t>17-08-2025</t>
         </is>
       </c>
       <c r="B201" s="1" t="inlineStr">
@@ -6467,7 +6467,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>15-08-2025</t>
+          <t>16-08-2025</t>
         </is>
       </c>
       <c r="B202" s="1" t="inlineStr">
@@ -6497,7 +6497,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>15-08-2025</t>
         </is>
       </c>
       <c r="B203" s="1" t="inlineStr">
@@ -6527,7 +6527,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>13-08-2025</t>
+          <t>14-08-2025</t>
         </is>
       </c>
       <c r="B204" s="1" t="inlineStr">
@@ -6541,23 +6541,23 @@
         </is>
       </c>
       <c r="D204" s="2" t="n">
-        <v>267.25</v>
+        <v>269.25</v>
       </c>
       <c r="E204" s="1" t="inlineStr">
         <is>
-          <t>13.08.2025</t>
+          <t>14.08.2025</t>
         </is>
       </c>
       <c r="F204" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>12-08-2025</t>
+          <t>13-08-2025</t>
         </is>
       </c>
       <c r="B205" s="1" t="inlineStr">
@@ -6571,23 +6571,23 @@
         </is>
       </c>
       <c r="D205" s="2" t="n">
-        <v>265.25</v>
+        <v>267.25</v>
       </c>
       <c r="E205" s="1" t="inlineStr">
         <is>
-          <t>12.08.2025</t>
+          <t>13.08.2025</t>
         </is>
       </c>
       <c r="F205" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>11-08-2025</t>
+          <t>12-08-2025</t>
         </is>
       </c>
       <c r="B206" s="1" t="inlineStr">
@@ -6601,23 +6601,23 @@
         </is>
       </c>
       <c r="D206" s="2" t="n">
-        <v>268.5</v>
+        <v>265.25</v>
       </c>
       <c r="E206" s="1" t="inlineStr">
         <is>
-          <t>08.08.2025</t>
+          <t>12.08.2025</t>
         </is>
       </c>
       <c r="F206" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>10-08-2025</t>
+          <t>11-08-2025</t>
         </is>
       </c>
       <c r="B207" s="1" t="inlineStr">
@@ -6647,7 +6647,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>09-08-2025</t>
+          <t>10-08-2025</t>
         </is>
       </c>
       <c r="B208" s="1" t="inlineStr">
@@ -6677,7 +6677,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>08-08-2025</t>
+          <t>09-08-2025</t>
         </is>
       </c>
       <c r="B209" s="1" t="inlineStr">
@@ -6707,7 +6707,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>07-08-2025</t>
+          <t>08-08-2025</t>
         </is>
       </c>
       <c r="B210" s="1" t="inlineStr">
@@ -6721,23 +6721,23 @@
         </is>
       </c>
       <c r="D210" s="2" t="n">
-        <v>265.75</v>
+        <v>268.5</v>
       </c>
       <c r="E210" s="1" t="inlineStr">
         <is>
-          <t>07.08.2025</t>
+          <t>08.08.2025</t>
         </is>
       </c>
       <c r="F210" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-08-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>06-08-2025</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="B211" s="1" t="inlineStr">
@@ -6751,23 +6751,23 @@
         </is>
       </c>
       <c r="D211" s="2" t="n">
-        <v>263.75</v>
+        <v>265.75</v>
       </c>
       <c r="E211" s="1" t="inlineStr">
         <is>
-          <t>05.08.2025</t>
+          <t>07.08.2025</t>
         </is>
       </c>
       <c r="F211" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>05-08-2025</t>
+          <t>06-08-2025</t>
         </is>
       </c>
       <c r="B212" s="1" t="inlineStr">
@@ -6797,7 +6797,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>04-08-2025</t>
+          <t>05-08-2025</t>
         </is>
       </c>
       <c r="B213" s="1" t="inlineStr">
@@ -6811,23 +6811,23 @@
         </is>
       </c>
       <c r="D213" s="2" t="n">
-        <v>260.5</v>
+        <v>263.75</v>
       </c>
       <c r="E213" s="1" t="inlineStr">
         <is>
-          <t>02.08.2025</t>
+          <t>05.08.2025</t>
         </is>
       </c>
       <c r="F213" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>03-08-2025</t>
+          <t>04-08-2025</t>
         </is>
       </c>
       <c r="B214" s="1" t="inlineStr">
@@ -6857,7 +6857,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>02-08-2025</t>
+          <t>03-08-2025</t>
         </is>
       </c>
       <c r="B215" s="1" t="inlineStr">
@@ -6887,7 +6887,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>01-08-2025</t>
+          <t>02-08-2025</t>
         </is>
       </c>
       <c r="B216" s="1" t="inlineStr">
@@ -6901,23 +6901,23 @@
         </is>
       </c>
       <c r="D216" s="2" t="n">
-        <v>264.5</v>
+        <v>260.5</v>
       </c>
       <c r="E216" s="1" t="inlineStr">
         <is>
-          <t>01.08.2025</t>
+          <t>02.08.2025</t>
         </is>
       </c>
       <c r="F216" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>31-07-2025</t>
+          <t>01-08-2025</t>
         </is>
       </c>
       <c r="B217" s="1" t="inlineStr">
@@ -6931,23 +6931,23 @@
         </is>
       </c>
       <c r="D217" s="2" t="n">
-        <v>266.25</v>
+        <v>264.5</v>
       </c>
       <c r="E217" s="1" t="inlineStr">
         <is>
-          <t>29.07.2025</t>
+          <t>01.08.2025</t>
         </is>
       </c>
       <c r="F217" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-august-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>30-07-2025</t>
+          <t>31-07-2025</t>
         </is>
       </c>
       <c r="B218" s="1" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>29-07-2025</t>
+          <t>30-07-2025</t>
         </is>
       </c>
       <c r="B219" s="1" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>28-07-2025</t>
+          <t>29-07-2025</t>
         </is>
       </c>
       <c r="B220" s="1" t="inlineStr">
@@ -7021,23 +7021,23 @@
         </is>
       </c>
       <c r="D220" s="2" t="n">
-        <v>268.5</v>
+        <v>266.25</v>
       </c>
       <c r="E220" s="1" t="inlineStr">
         <is>
-          <t>26.07.2025</t>
+          <t>29.07.2025</t>
         </is>
       </c>
       <c r="F220" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>27-07-2025</t>
+          <t>28-07-2025</t>
         </is>
       </c>
       <c r="B221" s="1" t="inlineStr">
@@ -7067,7 +7067,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>26-07-2025</t>
+          <t>27-07-2025</t>
         </is>
       </c>
       <c r="B222" s="1" t="inlineStr">
@@ -7097,7 +7097,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>25-07-2025</t>
+          <t>26-07-2025</t>
         </is>
       </c>
       <c r="B223" s="1" t="inlineStr">
@@ -7111,23 +7111,23 @@
         </is>
       </c>
       <c r="D223" s="2" t="n">
-        <v>267</v>
+        <v>268.5</v>
       </c>
       <c r="E223" s="1" t="inlineStr">
         <is>
-          <t>22.07.2025</t>
+          <t>26.07.2025</t>
         </is>
       </c>
       <c r="F223" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>24-07-2025</t>
+          <t>25-07-2025</t>
         </is>
       </c>
       <c r="B224" s="1" t="inlineStr">
@@ -7157,7 +7157,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>23-07-2025</t>
+          <t>24-07-2025</t>
         </is>
       </c>
       <c r="B225" s="1" t="inlineStr">
@@ -7187,7 +7187,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>22-07-2025</t>
+          <t>23-07-2025</t>
         </is>
       </c>
       <c r="B226" s="1" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>21-07-2025</t>
+          <t>22-07-2025</t>
         </is>
       </c>
       <c r="B227" s="1" t="inlineStr">
@@ -7231,23 +7231,23 @@
         </is>
       </c>
       <c r="D227" s="2" t="n">
-        <v>261.5</v>
+        <v>267</v>
       </c>
       <c r="E227" s="1" t="inlineStr">
         <is>
-          <t>19.07.2025</t>
+          <t>22.07.2025</t>
         </is>
       </c>
       <c r="F227" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-22-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>21-07-2025</t>
         </is>
       </c>
       <c r="B228" s="1" t="inlineStr">
@@ -7277,7 +7277,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>19-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="B229" s="1" t="inlineStr">
@@ -7307,7 +7307,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>18-07-2025</t>
+          <t>19-07-2025</t>
         </is>
       </c>
       <c r="B230" s="1" t="inlineStr">
@@ -7321,23 +7321,23 @@
         </is>
       </c>
       <c r="D230" s="2" t="n">
-        <v>258</v>
+        <v>261.5</v>
       </c>
       <c r="E230" s="1" t="inlineStr">
         <is>
-          <t>17.07.2025</t>
+          <t>19.07.2025</t>
         </is>
       </c>
       <c r="F230" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>17-07-2025</t>
+          <t>18-07-2025</t>
         </is>
       </c>
       <c r="B231" s="1" t="inlineStr">
@@ -7367,7 +7367,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>16-07-2025</t>
+          <t>17-07-2025</t>
         </is>
       </c>
       <c r="B232" s="1" t="inlineStr">
@@ -7381,23 +7381,23 @@
         </is>
       </c>
       <c r="D232" s="2" t="n">
-        <v>261.25</v>
+        <v>258</v>
       </c>
       <c r="E232" s="1" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="F232" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>15-07-2025</t>
+          <t>16-07-2025</t>
         </is>
       </c>
       <c r="B233" s="1" t="inlineStr">
@@ -7427,7 +7427,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>14-07-2025</t>
+          <t>15-07-2025</t>
         </is>
       </c>
       <c r="B234" s="1" t="inlineStr">
@@ -7457,7 +7457,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>13-07-2025</t>
+          <t>14-07-2025</t>
         </is>
       </c>
       <c r="B235" s="1" t="inlineStr">
@@ -7487,7 +7487,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>12-07-2025</t>
+          <t>13-07-2025</t>
         </is>
       </c>
       <c r="B236" s="1" t="inlineStr">
@@ -7517,7 +7517,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>11-07-2025</t>
+          <t>12-07-2025</t>
         </is>
       </c>
       <c r="B237" s="1" t="inlineStr">
@@ -7547,7 +7547,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>10-07-2025</t>
+          <t>11-07-2025</t>
         </is>
       </c>
       <c r="B238" s="1" t="inlineStr">
@@ -7561,23 +7561,23 @@
         </is>
       </c>
       <c r="D238" s="2" t="n">
-        <v>258.5</v>
+        <v>261.25</v>
       </c>
       <c r="E238" s="1" t="inlineStr">
         <is>
-          <t>05.07.2025</t>
+          <t>11.07.2025</t>
         </is>
       </c>
       <c r="F238" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>09-07-2025</t>
+          <t>10-07-2025</t>
         </is>
       </c>
       <c r="B239" s="1" t="inlineStr">
@@ -7607,7 +7607,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>08-07-2025</t>
+          <t>09-07-2025</t>
         </is>
       </c>
       <c r="B240" s="1" t="inlineStr">
@@ -7637,7 +7637,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>07-07-2025</t>
+          <t>08-07-2025</t>
         </is>
       </c>
       <c r="B241" s="1" t="inlineStr">
@@ -7667,7 +7667,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>06-07-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="B242" s="1" t="inlineStr">
@@ -7697,7 +7697,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>05-07-2025</t>
+          <t>06-07-2025</t>
         </is>
       </c>
       <c r="B243" s="1" t="inlineStr">
@@ -7727,7 +7727,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>04-07-2025</t>
+          <t>05-07-2025</t>
         </is>
       </c>
       <c r="B244" s="1" t="inlineStr">
@@ -7741,23 +7741,23 @@
         </is>
       </c>
       <c r="D244" s="2" t="n">
-        <v>260.75</v>
+        <v>258.5</v>
       </c>
       <c r="E244" s="1" t="inlineStr">
         <is>
-          <t>02.07.2025</t>
+          <t>05.07.2025</t>
         </is>
       </c>
       <c r="F244" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>04-07-2025</t>
         </is>
       </c>
       <c r="B245" s="1" t="inlineStr">
@@ -7787,7 +7787,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>02-07-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="B246" s="1" t="inlineStr">
@@ -7817,7 +7817,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>01-07-2025</t>
+          <t>02-07-2025</t>
         </is>
       </c>
       <c r="B247" s="1" t="inlineStr">
@@ -7831,23 +7831,23 @@
         </is>
       </c>
       <c r="D247" s="2" t="n">
-        <v>263.25</v>
+        <v>260.75</v>
       </c>
       <c r="E247" s="1" t="inlineStr">
         <is>
-          <t>28.06.2025</t>
+          <t>02.07.2025</t>
         </is>
       </c>
       <c r="F247" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-02-july-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>30-06-2025</t>
+          <t>01-07-2025</t>
         </is>
       </c>
       <c r="B248" s="1" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>29-06-2025</t>
+          <t>30-06-2025</t>
         </is>
       </c>
       <c r="B249" s="1" t="inlineStr">
@@ -7907,7 +7907,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>28-06-2025</t>
+          <t>29-06-2025</t>
         </is>
       </c>
       <c r="B250" s="1" t="inlineStr">
@@ -7937,7 +7937,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>27-06-2025</t>
+          <t>28-06-2025</t>
         </is>
       </c>
       <c r="B251" s="1" t="inlineStr">
@@ -7951,23 +7951,23 @@
         </is>
       </c>
       <c r="D251" s="2" t="n">
-        <v>261.75</v>
+        <v>263.25</v>
       </c>
       <c r="E251" s="1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>28.06.2025</t>
         </is>
       </c>
       <c r="F251" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>26-06-2025</t>
+          <t>27-06-2025</t>
         </is>
       </c>
       <c r="B252" s="1" t="inlineStr">
@@ -7997,7 +7997,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>25-06-2025</t>
+          <t>26-06-2025</t>
         </is>
       </c>
       <c r="B253" s="1" t="inlineStr">
@@ -8011,23 +8011,23 @@
         </is>
       </c>
       <c r="D253" s="2" t="n">
-        <v>264</v>
+        <v>261.75</v>
       </c>
       <c r="E253" s="1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="F253" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>24-06-2025</t>
+          <t>25-06-2025</t>
         </is>
       </c>
       <c r="B254" s="1" t="inlineStr">
@@ -8041,23 +8041,23 @@
         </is>
       </c>
       <c r="D254" s="2" t="n">
-        <v>268.75</v>
+        <v>264</v>
       </c>
       <c r="E254" s="1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="F254" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>23-06-2025</t>
+          <t>24-06-2025</t>
         </is>
       </c>
       <c r="B255" s="1" t="inlineStr">
@@ -8071,23 +8071,23 @@
         </is>
       </c>
       <c r="D255" s="2" t="n">
-        <v>262.25</v>
+        <v>268.75</v>
       </c>
       <c r="E255" s="1" t="inlineStr">
         <is>
-          <t>19.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F255" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>23-06-2025</t>
         </is>
       </c>
       <c r="B256" s="1" t="inlineStr">
@@ -8117,7 +8117,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>21-06-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="B257" s="1" t="inlineStr">
@@ -8147,7 +8147,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>20-06-2025</t>
+          <t>21-06-2025</t>
         </is>
       </c>
       <c r="B258" s="1" t="inlineStr">
@@ -8177,7 +8177,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>19-06-2025</t>
+          <t>20-06-2025</t>
         </is>
       </c>
       <c r="B259" s="1" t="inlineStr">
@@ -8207,7 +8207,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>18-06-2025</t>
+          <t>19-06-2025</t>
         </is>
       </c>
       <c r="B260" s="1" t="inlineStr">
@@ -8221,23 +8221,23 @@
         </is>
       </c>
       <c r="D260" s="2" t="n">
-        <v>260</v>
+        <v>262.25</v>
       </c>
       <c r="E260" s="1" t="inlineStr">
         <is>
-          <t>18.06.2025</t>
+          <t>19.06.2025</t>
         </is>
       </c>
       <c r="F260" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>17-06-2025</t>
+          <t>18-06-2025</t>
         </is>
       </c>
       <c r="B261" s="1" t="inlineStr">
@@ -8251,23 +8251,23 @@
         </is>
       </c>
       <c r="D261" s="2" t="n">
-        <v>256.5</v>
+        <v>260</v>
       </c>
       <c r="E261" s="1" t="inlineStr">
         <is>
-          <t>12.06.2025</t>
+          <t>18.06.2025</t>
         </is>
       </c>
       <c r="F261" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-june-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>17-06-2025</t>
         </is>
       </c>
       <c r="B262" s="1" t="inlineStr">
@@ -8297,7 +8297,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>15-06-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="B263" s="1" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>14-06-2025</t>
+          <t>15-06-2025</t>
         </is>
       </c>
       <c r="B264" s="1" t="inlineStr">
@@ -8357,7 +8357,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>13-06-2025</t>
+          <t>14-06-2025</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
@@ -8387,7 +8387,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>12-06-2025</t>
+          <t>13-06-2025</t>
         </is>
       </c>
       <c r="B266" s="1" t="inlineStr">
@@ -8409,6 +8409,36 @@
         </is>
       </c>
       <c r="F266" s="1" t="inlineStr">
+        <is>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="1" t="inlineStr">
+        <is>
+          <t>12-06-2025</t>
+        </is>
+      </c>
+      <c r="B267" s="1" t="inlineStr">
+        <is>
+          <t>2. P0610 (99.85% min) /P1020/ EC Grade Ingot &amp; Sow 99.7% (min) / Cast Bar</t>
+        </is>
+      </c>
+      <c r="C267" s="1" t="inlineStr">
+        <is>
+          <t>P1020</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="n">
+        <v>256.5</v>
+      </c>
+      <c r="E267" s="1" t="inlineStr">
+        <is>
+          <t>12.06.2025</t>
+        </is>
+      </c>
+      <c r="F267" s="1" t="inlineStr">
         <is>
           <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-june-2025.pdf</t>
         </is>
@@ -8681,6 +8711,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId263"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId264"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F267" r:id="rId266"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hindalco: update PDFs & Excel (2026-03-05 03:14:23 UTC)
</commit_message>
<xml_diff>
--- a/data/hindalco_prices.xlsx
+++ b/data/hindalco_prices.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F267"/>
+  <dimension ref="A1:F268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>04-03-2026</t>
+          <t>05-03-2026</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>03-03-2026</t>
+          <t>04-03-2026</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>02-03-2026</t>
+          <t>03-03-2026</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -541,23 +541,23 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>338.25</v>
+        <v>346.75</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>28.02.2026</t>
+          <t>03.03.2026</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-march-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>01-03-2026</t>
+          <t>02-03-2026</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>28-02-2026</t>
+          <t>01-03-2026</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>27-02-2026</t>
+          <t>28-02-2026</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -631,23 +631,23 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>334.5</v>
+        <v>338.25</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>27.02.2026</t>
+          <t>28.02.2026</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-28-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>27-02-2026</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -661,23 +661,23 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>333.25</v>
+        <v>334.5</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>26.02.2026</t>
+          <t>27.02.2026</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-27-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>25-02-2026</t>
+          <t>26-02-2026</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -691,23 +691,23 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>330.5</v>
+        <v>333.25</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>25.02.2026</t>
+          <t>26.02.2026</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-26-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>24-02-2026</t>
+          <t>25-02-2026</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>328.25</v>
+        <v>330.5</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>21.02.2026</t>
+          <t>25.02.2026</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>23-02-2026</t>
+          <t>24-02-2026</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>22-02-2026</t>
+          <t>23-02-2026</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -797,7 +797,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>21-02-2026</t>
+          <t>22-02-2026</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>20-02-2026</t>
+          <t>21-02-2026</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -841,23 +841,23 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>325.75</v>
+        <v>328.25</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>19.02.2026</t>
+          <t>21.02.2026</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>19-02-2026</t>
+          <t>20-02-2026</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>18-02-2026</t>
+          <t>19-02-2026</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -901,23 +901,23 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>324</v>
+        <v>325.75</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>18.02.2026</t>
+          <t>19.02.2026</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-19-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>17-02-2026</t>
+          <t>18-02-2026</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -931,23 +931,23 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>326.25</v>
+        <v>324</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
-          <t>17.02.2026</t>
+          <t>18.02.2026</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-18-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>16-02-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
@@ -961,23 +961,23 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>322.5</v>
+        <v>326.25</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>14.02.2026</t>
+          <t>17.02.2026</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>15-02-2026</t>
+          <t>16-02-2026</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>14-02-2026</t>
+          <t>15-02-2026</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>13-02-2026</t>
+          <t>14-02-2026</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
@@ -1051,23 +1051,23 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>334</v>
+        <v>322.5</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>13.02.2026</t>
+          <t>14.02.2026</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>13-02-2026</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
@@ -1081,23 +1081,23 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>12.02.2026</t>
+          <t>13.02.2026</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1111,23 +1111,23 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>328.75</v>
+        <v>332</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>11.02.2026</t>
+          <t>12.02.2026</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-12-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>10-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
@@ -1141,23 +1141,23 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>330.25</v>
+        <v>328.75</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>10.02.2026</t>
+          <t>11.02.2026</t>
         </is>
       </c>
       <c r="F24" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-11-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>09-02-2026</t>
+          <t>10-02-2026</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1171,23 +1171,23 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>326.5</v>
+        <v>330.25</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>10.02.2026</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>08-02-2026</t>
+          <t>09-02-2026</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>07-02-2026</t>
+          <t>08-02-2026</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>06-02-2026</t>
+          <t>07-02-2026</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1261,23 +1261,23 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>323.5</v>
+        <v>326.5</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>06.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>05-02-2026</t>
+          <t>06-02-2026</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
@@ -1291,23 +1291,23 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>327</v>
+        <v>323.5</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>05.02.2026</t>
+          <t>06.02.2026</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>04-02-2026</t>
+          <t>05-02-2026</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1321,23 +1321,23 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>332.25</v>
+        <v>327</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>04.02.2026</t>
+          <t>05.02.2026</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-05-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>03-02-2026</t>
+          <t>04-02-2026</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1351,23 +1351,23 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>330.75</v>
+        <v>332.25</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>03.02.2026</t>
+          <t>04.02.2026</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-04-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>02-02-2026</t>
+          <t>03-02-2026</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
@@ -1381,23 +1381,23 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>338.25</v>
+        <v>330.75</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>31.01.2026</t>
+          <t>03.02.2026</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-february-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>01-02-2026</t>
+          <t>02-02-2026</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>31-01-2026</t>
+          <t>01-02-2026</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>30-01-2026</t>
+          <t>31-01-2026</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
@@ -1471,23 +1471,23 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>360</v>
+        <v>338.25</v>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
+          <t>31.01.2026</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>29-01-2026</t>
+          <t>30-01-2026</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
@@ -1501,23 +1501,23 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>352.25</v>
+        <v>360</v>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>29.01.2026</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-30-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>28-01-2026</t>
+          <t>29-01-2026</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1531,23 +1531,23 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>343.5</v>
+        <v>352.25</v>
       </c>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>24.01.2026</t>
+          <t>29.01.2026</t>
         </is>
       </c>
       <c r="F37" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-29-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>27-01-2026</t>
+          <t>28-01-2026</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
@@ -1577,7 +1577,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>27-01-2026</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>25-01-2026</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>24-01-2026</t>
+          <t>25-01-2026</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>23-01-2026</t>
+          <t>24-01-2026</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
@@ -1681,23 +1681,23 @@
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>335.5</v>
+        <v>343.5</v>
       </c>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>21.01.2026</t>
+          <t>24.01.2026</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>22-01-2026</t>
+          <t>23-01-2026</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>21-01-2026</t>
+          <t>22-01-2026</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
@@ -1757,7 +1757,7 @@
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>20-01-2026</t>
+          <t>21-01-2026</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
@@ -1771,23 +1771,23 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>338.5</v>
+        <v>335.5</v>
       </c>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>20.01.2026</t>
+          <t>21.01.2026</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-21-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>19-01-2026</t>
+          <t>20-01-2026</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1801,23 +1801,23 @@
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>335</v>
+        <v>338.5</v>
       </c>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>17.01.2026</t>
+          <t>20.01.2026</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>18-01-2026</t>
+          <t>19-01-2026</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>17-01-2026</t>
+          <t>18-01-2026</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>16-01-2026</t>
+          <t>17-01-2026</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
@@ -1891,23 +1891,23 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>343.25</v>
+        <v>335</v>
       </c>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>15.01.2026</t>
+          <t>17.01.2026</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>15-01-2026</t>
+          <t>16-01-2026</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>14-01-2026</t>
+          <t>15-01-2026</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
@@ -1951,23 +1951,23 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>340.75</v>
+        <v>343.25</v>
       </c>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>14.01.2026</t>
+          <t>15.01.2026</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-15-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>13-01-2026</t>
+          <t>14-01-2026</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
@@ -1981,23 +1981,23 @@
         </is>
       </c>
       <c r="D52" s="2" t="n">
-        <v>338.75</v>
+        <v>340.75</v>
       </c>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>10.01.2026</t>
+          <t>14.01.2026</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-14-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>12-01-2026</t>
+          <t>13-01-2026</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>11-01-2026</t>
+          <t>12-01-2026</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
@@ -2057,7 +2057,7 @@
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>10-01-2026</t>
+          <t>11-01-2026</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>09-01-2026</t>
+          <t>10-01-2026</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
@@ -2101,23 +2101,23 @@
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>328</v>
+        <v>338.75</v>
       </c>
       <c r="E56" s="1" t="inlineStr">
         <is>
-          <t>09.01.2026</t>
+          <t>10.01.2026</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-10-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>08-01-2026</t>
+          <t>09-01-2026</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
@@ -2131,23 +2131,23 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E57" s="1" t="inlineStr">
         <is>
-          <t>07.01.2026</t>
+          <t>09.01.2026</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-09-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>07-01-2026</t>
+          <t>08-01-2026</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
@@ -2177,7 +2177,7 @@
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>06-01-2026</t>
+          <t>07-01-2026</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
@@ -2191,23 +2191,23 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>323.25</v>
+        <v>330</v>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>06.01.2026</t>
+          <t>07.01.2026</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-07-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>05-01-2026</t>
+          <t>06-01-2026</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
@@ -2221,23 +2221,23 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>319.25</v>
+        <v>323.25</v>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>03.01.2026</t>
+          <t>06.01.2026</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-06-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>04-01-2026</t>
+          <t>05-01-2026</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>03-01-2026</t>
+          <t>04-01-2026</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
@@ -2297,7 +2297,7 @@
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>02-01-2026</t>
+          <t>03-01-2026</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
@@ -2311,23 +2311,23 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>316.75</v>
+        <v>319.25</v>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>01.01.2026</t>
+          <t>03.01.2026</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-03-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>01-01-2026</t>
+          <t>02-01-2026</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>31-12-2025</t>
+          <t>01-01-2026</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
@@ -2371,23 +2371,23 @@
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>314.5</v>
+        <v>316.75</v>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>31.12.2025</t>
+          <t>01.01.2026</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-01-january-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>30-12-2025</t>
+          <t>31-12-2025</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
@@ -2401,23 +2401,23 @@
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>312.5</v>
+        <v>314.5</v>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>25.12.2025</t>
+          <t>31.12.2025</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-31-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>29-12-2025</t>
+          <t>30-12-2025</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>28-12-2025</t>
+          <t>29-12-2025</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
@@ -2477,7 +2477,7 @@
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>27-12-2025</t>
+          <t>28-12-2025</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>26-12-2025</t>
+          <t>27-12-2025</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
@@ -2537,7 +2537,7 @@
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>25-12-2025</t>
+          <t>26-12-2025</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>24-12-2025</t>
+          <t>25-12-2025</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
@@ -2581,23 +2581,23 @@
         </is>
       </c>
       <c r="D72" s="2" t="n">
-        <v>310.75</v>
+        <v>312.5</v>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>24.12.2025</t>
+          <t>25.12.2025</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-25-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>23-12-2025</t>
+          <t>24-12-2025</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
@@ -2611,23 +2611,23 @@
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>307.25</v>
+        <v>310.75</v>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>23.12.2025</t>
+          <t>24.12.2025</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-24-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>22-12-2025</t>
+          <t>23-12-2025</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
@@ -2641,23 +2641,23 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>309.25</v>
+        <v>307.25</v>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>20.12.2025</t>
+          <t>23.12.2025</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-23-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>21-12-2025</t>
+          <t>22-12-2025</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>20-12-2025</t>
+          <t>21-12-2025</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>19-12-2025</t>
+          <t>20-12-2025</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
@@ -2731,23 +2731,23 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>304.5</v>
+        <v>309.25</v>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>17.12.2025</t>
+          <t>20.12.2025</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-20-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>18-12-2025</t>
+          <t>19-12-2025</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
@@ -2777,7 +2777,7 @@
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>17-12-2025</t>
+          <t>18-12-2025</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>16-12-2025</t>
+          <t>17-12-2025</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
@@ -2821,23 +2821,23 @@
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>303</v>
+        <v>304.5</v>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>13.12.2025</t>
+          <t>17.12.2025</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-13-december-2025.pdf</t>
+          <t>https://www.hindalco.com/Upload/PDF/primary-ready-reckoner-17-december-2025.pdf</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>15-12-2025</t>
+          <t>16-12-2025</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>14-12-2025</t>
+          <t>15-